<commit_message>
EA dataset fixed FG shock scaling fixed .
</commit_message>
<xml_diff>
--- a/irf/irf/Paper IRFs.xlsx
+++ b/irf/irf/Paper IRFs.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
   <si>
     <t>t</t>
   </si>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <t>2025-12-18T15:29:26.11</t>
+  </si>
+  <si>
+    <t>2026-02-10T13:49:09.578</t>
+  </si>
+  <si>
+    <t>2026-02-10T13:51:34.338</t>
   </si>
 </sst>
 </file>
@@ -501,13 +507,13 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="J1" t="s">
         <v>8</v>
       </c>
       <c r="K1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -533,7 +539,7 @@
         <v>2.5793795815169456</v>
       </c>
       <c r="H2">
-        <v>-6.355787355569827e-15</v>
+        <v>-1.0776287571287195</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -559,7 +565,7 @@
         <v>1.4953394328181018</v>
       </c>
       <c r="H3">
-        <v>-1.6480533826595375e-15</v>
+        <v>-1.0901798523912853</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -585,7 +591,7 @@
         <v>1.1447890872423834</v>
       </c>
       <c r="H4">
-        <v>-2.081899328946869e-15</v>
+        <v>-1.1050722210876067</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -611,7 +617,7 @@
         <v>0.9056919935333063</v>
       </c>
       <c r="H5">
-        <v>-1.6504474741377359e-15</v>
+        <v>-1.1161558581396847</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -637,7 +643,7 @@
         <v>0.7319914235132261</v>
       </c>
       <c r="H6">
-        <v>-1.0682857281982889e-15</v>
+        <v>-1.124275171477677</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -663,7 +669,7 @@
         <v>0.5973427245187732</v>
       </c>
       <c r="H7">
-        <v>-3.351537685000903e-16</v>
+        <v>-1.1300125312110396</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -689,7 +695,7 @@
         <v>-0.1711148877063895</v>
       </c>
       <c r="H8">
-        <v>2.1604510794098216e-15</v>
+        <v>-0.8589162460761607</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -715,7 +721,7 @@
         <v>-0.48020139575093257</v>
       </c>
       <c r="H9">
-        <v>3.1695275586680018e-15</v>
+        <v>-0.6527917857811548</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -741,7 +747,7 @@
         <v>-0.5768324684811983</v>
       </c>
       <c r="H10">
-        <v>4.25340167117954e-15</v>
+        <v>-0.518379630721563</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -767,7 +773,7 @@
         <v>-0.5871768624011784</v>
       </c>
       <c r="H11">
-        <v>5.334502974659489e-15</v>
+        <v>-0.4302230951401023</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -793,7 +799,7 @@
         <v>-0.5655516135502099</v>
       </c>
       <c r="H12">
-        <v>6.374359255433715e-15</v>
+        <v>-0.37025101988486603</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -819,7 +825,7 @@
         <v>-0.5334958471292568</v>
       </c>
       <c r="H13">
-        <v>7.348022928166114e-15</v>
+        <v>-0.32798101284319414</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -845,7 +851,7 @@
         <v>-0.499029394560659</v>
       </c>
       <c r="H14">
-        <v>8.238600942484928e-15</v>
+        <v>-0.29728557226249874</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -871,7 +877,7 @@
         <v>-0.46490712897908937</v>
       </c>
       <c r="H15">
-        <v>9.035400836782848e-15</v>
+        <v>-0.27435118561052385</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -897,7 +903,7 @@
         <v>-0.43193786324030503</v>
       </c>
       <c r="H16">
-        <v>9.732723232297122e-15</v>
+        <v>-0.2566500422596416</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -923,7 +929,7 @@
         <v>-0.4002656212734461</v>
       </c>
       <c r="H17">
-        <v>1.0328839915493663e-14</v>
+        <v>-0.24243423152081073</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -949,7 +955,7 @@
         <v>-0.3698442820958281</v>
       </c>
       <c r="H18">
-        <v>1.0825107183252934e-14</v>
+        <v>-0.23047147775076154</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -975,7 +981,7 @@
         <v>-0.34060187362750494</v>
       </c>
       <c r="H19">
-        <v>1.1225210005760732e-14</v>
+        <v>-0.2198922430955447</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -1001,7 +1007,7 @@
         <v>-0.31248901919794614</v>
       </c>
       <c r="H20">
-        <v>1.1534528912238757e-14</v>
+        <v>-0.21009142183175822</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -1027,7 +1033,7 @@
         <v>-0.2854862761513888</v>
       </c>
       <c r="H21">
-        <v>1.175961705074767e-14</v>
+        <v>-0.20065974270055495</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -1053,7 +1059,7 @@
         <v>-0.259598482828578</v>
       </c>
       <c r="H22">
-        <v>1.1907773598333052e-14</v>
+        <v>-0.19133336646627905</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -1079,7 +1085,7 @@
         <v>-0.23484632667295546</v>
       </c>
       <c r="H23">
-        <v>1.198670019418404e-14</v>
+        <v>-0.1819558083010112</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -1105,7 +1111,7 @@
         <v>-0.2112585709882856</v>
       </c>
       <c r="H24">
-        <v>1.2004228239577581e-14</v>
+        <v>-0.1724488035363658</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -1131,7 +1137,7 @@
         <v>-0.18886587385927223</v>
       </c>
       <c r="H25">
-        <v>1.1968106244614112e-14</v>
+        <v>-0.16278992968392045</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -1157,7 +1163,7 @@
         <v>-0.1676962516278695</v>
       </c>
       <c r="H26">
-        <v>1.188583770482846e-14</v>
+        <v>-0.15299544177405125</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -1183,7 +1189,7 @@
         <v>-0.14777196505869047</v>
       </c>
       <c r="H27">
-        <v>1.1764561194408282e-14</v>
+        <v>-0.14310717159366784</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -1209,7 +1215,7 @@
         <v>-0.12910755184239306</v>
       </c>
       <c r="H28">
-        <v>1.1610965451139909e-14</v>
+        <v>-0.1331826081151621</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -1235,7 +1241,7 @@
         <v>-0.11170874851067299</v>
       </c>
       <c r="H29">
-        <v>1.1431233203186396e-14</v>
+        <v>-0.12328747034328749</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -1261,7 +1267,7 @@
         <v>-0.09557208436693596</v>
       </c>
       <c r="H30">
-        <v>1.1231008356708719e-14</v>
+        <v>-0.11349023077698193</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -1287,7 +1293,7 @@
         <v>-0.08068497073909373</v>
       </c>
       <c r="H31">
-        <v>1.1015381934708296e-14</v>
+        <v>-0.10385816158716517</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -1313,7 +1319,7 @@
         <v>-0.06702614481783115</v>
       </c>
       <c r="H32">
-        <v>1.0788892839714788e-14</v>
+        <v>-0.09445456493197307</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -1339,7 +1345,7 @@
         <v>-0.05456635734818738</v>
       </c>
       <c r="H33">
-        <v>1.0555540114031386e-14</v>
+        <v>-0.08533691930916376</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -1365,7 +1371,7 @@
         <v>-0.0432692178717905</v>
       </c>
       <c r="H34">
-        <v>1.031880389865131e-14</v>
+        <v>-0.07655572964759738</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -1391,7 +1397,7 @@
         <v>-0.03309213088256757</v>
       </c>
       <c r="H35">
-        <v>1.0081672752685079e-14</v>
+        <v>-0.0681539131143121</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -1417,7 +1423,7 @@
         <v>-0.02398727199936468</v>
       </c>
       <c r="H36">
-        <v>9.84667539576943e-15</v>
+        <v>-0.06016658779289161</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -1443,7 +1449,7 @@
         <v>-0.015902565816211744</v>
       </c>
       <c r="H37">
-        <v>9.61591528263049e-15</v>
+        <v>-0.0526211593726106</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -1469,7 +1475,7 @@
         <v>-0.00878263708310384</v>
       </c>
       <c r="H38">
-        <v>9.391106717500169e-15</v>
+        <v>-0.04553762326926426</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -1495,7 +1501,7 @@
         <v>-0.002569714800012668</v>
       </c>
       <c r="H39">
-        <v>9.173611471779087e-15</v>
+        <v>-0.03892901735440936</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -1521,7 +1527,7 @@
         <v>0.002795524920532755</v>
       </c>
       <c r="H40">
-        <v>8.964475086133226e-15</v>
+        <v>-0.03280197462915188</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -1547,7 +1553,7 @@
         <v>0.007373186426717637</v>
       </c>
       <c r="H41">
-        <v>8.764462222628797e-15</v>
+        <v>-0.02715733647615541</v>
       </c>
     </row>
   </sheetData>
@@ -1571,19 +1577,19 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F1" t="s">
         <v>20</v>
       </c>
       <c r="G1" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="H1" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="J1" t="s">
         <v>8</v>
@@ -1597,16 +1603,16 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>-3.4528186345588288</v>
+        <v>8.102500031716193</v>
       </c>
       <c r="C2">
         <v>0.0</v>
       </c>
       <c r="D2">
-        <v>-1.0000000000000002</v>
+        <v>-1.0</v>
       </c>
       <c r="E2">
-        <v>-0.6724381448767072</v>
+        <v>0.3002694365653483</v>
       </c>
       <c r="F2">
         <v>-1.8240941779797443e-14</v>
@@ -1623,7 +1629,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>-2.2470266251559217</v>
+        <v>3.7924900644128168</v>
       </c>
       <c r="C3">
         <v>0.0</v>
@@ -1632,7 +1638,7 @@
         <v>-1.0</v>
       </c>
       <c r="E3">
-        <v>-0.6754920439440941</v>
+        <v>0.34132427283477856</v>
       </c>
       <c r="F3">
         <v>-1.815767595640473e-14</v>
@@ -1649,16 +1655,16 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>-1.620532378859584</v>
+        <v>1.535682253088882</v>
       </c>
       <c r="C4">
         <v>0.0</v>
       </c>
       <c r="D4">
-        <v>-1.0</v>
+        <v>-1.0000000000000002</v>
       </c>
       <c r="E4">
-        <v>-0.6914267332173135</v>
+        <v>0.3262395395059982</v>
       </c>
       <c r="F4">
         <v>-1.7990016981340348e-14</v>
@@ -1675,7 +1681,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>-1.2672896844330825</v>
+        <v>0.314417515476746</v>
       </c>
       <c r="C5">
         <v>0.0</v>
@@ -1684,7 +1690,7 @@
         <v>-1.0</v>
       </c>
       <c r="E5">
-        <v>-0.7126190796009902</v>
+        <v>0.297172637639562</v>
       </c>
       <c r="F5">
         <v>-1.7750026373046594e-14</v>
@@ -1701,16 +1707,16 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>-1.0342703989673754</v>
+        <v>-0.3714566512920629</v>
       </c>
       <c r="C6">
         <v>0.0</v>
       </c>
       <c r="D6">
-        <v>-0.9999999999999999</v>
+        <v>-1.0000000000000002</v>
       </c>
       <c r="E6">
-        <v>-0.7369490309361146</v>
+        <v>0.26450237048056346</v>
       </c>
       <c r="F6">
         <v>-1.7449311279723872e-14</v>
@@ -1727,7 +1733,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>-0.8446534793547582</v>
+        <v>-0.7682647916323465</v>
       </c>
       <c r="C7">
         <v>0.0</v>
@@ -1736,7 +1742,7 @@
         <v>-1.0</v>
       </c>
       <c r="E7">
-        <v>-0.7634137716033613</v>
+        <v>0.23168373759607122</v>
       </c>
       <c r="F7">
         <v>-1.7098845668544484e-14</v>
@@ -1753,16 +1759,16 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>-0.6587311709284003</v>
+        <v>-0.9983762771240359</v>
       </c>
       <c r="C8">
         <v>0.0</v>
       </c>
       <c r="D8">
-        <v>1.0018733440900038</v>
+        <v>-0.8228559440075205</v>
       </c>
       <c r="E8">
-        <v>1.2106152491219866</v>
+        <v>0.20029060488665273</v>
       </c>
       <c r="F8">
         <v>-1.6708846025861055e-14</v>
@@ -1779,16 +1785,16 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0.24680905953848103</v>
+        <v>-1.0615234494165005</v>
       </c>
       <c r="C9">
         <v>0.0</v>
       </c>
       <c r="D9">
-        <v>1.0184154340610958</v>
+        <v>-0.6802281125838083</v>
       </c>
       <c r="E9">
-        <v>1.1997204343437553</v>
+        <v>0.17117303992476582</v>
       </c>
       <c r="F9">
         <v>-1.628869161461582e-14</v>
@@ -1805,16 +1811,16 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>0.7263675921425222</v>
+        <v>-1.0428589933721009</v>
       </c>
       <c r="C10">
         <v>0.0</v>
       </c>
       <c r="D10">
-        <v>0.8156573832361733</v>
+        <v>-0.5839658177105793</v>
       </c>
       <c r="E10">
-        <v>0.9711631474977384</v>
+        <v>0.14469354968982942</v>
       </c>
       <c r="F10">
         <v>-1.5846880766101665e-14</v>
@@ -1831,16 +1837,16 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>0.8982855718353012</v>
+        <v>-0.9921377386601233</v>
       </c>
       <c r="C11">
         <v>0.0</v>
       </c>
       <c r="D11">
-        <v>0.6586264335291566</v>
+        <v>-0.5204572812941362</v>
       </c>
       <c r="E11">
-        <v>0.7905470542901465</v>
+        <v>0.1209314480216968</v>
       </c>
       <c r="F11">
         <v>-1.5391015939674246e-14</v>
@@ -1857,16 +1863,16 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0.9255227013030343</v>
+        <v>-0.9313171317033377</v>
       </c>
       <c r="C12">
         <v>0.0</v>
       </c>
       <c r="D12">
-        <v>0.5570036467058181</v>
+        <v>-0.4780823352039272</v>
       </c>
       <c r="E12">
-        <v>0.6677310999777817</v>
+        <v>0.0998197529172179</v>
       </c>
       <c r="F12">
         <v>-1.492781138475873e-14</v>
@@ -1883,16 +1889,16 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>0.8946469763358686</v>
+        <v>-0.8688979012157303</v>
       </c>
       <c r="C13">
         <v>0.0</v>
       </c>
       <c r="D13">
-        <v>0.49186589094678723</v>
+        <v>-0.44914320705740507</v>
       </c>
       <c r="E13">
-        <v>0.5837699848463117</v>
+        <v>0.08122018743975548</v>
       </c>
       <c r="F13">
         <v>-1.4463118201713377e-14</v>
@@ -1909,16 +1915,16 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>0.8432769678272334</v>
+        <v>-0.8077995380727517</v>
       </c>
       <c r="C14">
         <v>0.0</v>
       </c>
       <c r="D14">
-        <v>0.4488642256802755</v>
+        <v>-0.42862347099199605</v>
       </c>
       <c r="E14">
-        <v>0.5242002936670479</v>
+        <v>0.06496131838760792</v>
       </c>
       <c r="F14">
         <v>-1.4001962437076097e-14</v>
@@ -1935,16 +1941,16 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>0.7862841894323267</v>
+        <v>-0.7488403124163857</v>
       </c>
       <c r="C15">
         <v>0.0</v>
       </c>
       <c r="D15">
-        <v>0.4193036627477743</v>
+        <v>-0.41317369462819337</v>
       </c>
       <c r="E15">
-        <v>0.48017247947465613</v>
+        <v>0.05085802283127187</v>
       </c>
       <c r="F15">
         <v>-1.3548592577989773e-14</v>
@@ -1961,16 +1967,16 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>0.7291287172948163</v>
+        <v>-0.6921339810602081</v>
       </c>
       <c r="C16">
         <v>0.0</v>
       </c>
       <c r="D16">
-        <v>0.39794057515986725</v>
+        <v>-0.4005166921982795</v>
       </c>
       <c r="E16">
-        <v>0.44627304444263516</v>
+        <v>0.03872194353595661</v>
       </c>
       <c r="F16">
         <v>-1.3106533442287815e-14</v>
@@ -1987,16 +1993,16 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>0.6736313551308237</v>
+        <v>-0.6376112097334082</v>
       </c>
       <c r="C17">
         <v>0.0</v>
       </c>
       <c r="D17">
-        <v>0.3814757938431972</v>
+        <v>-0.38910425750694966</v>
       </c>
       <c r="E17">
-        <v>0.41902976580950124</v>
+        <v>0.028367498022029917</v>
       </c>
       <c r="F17">
         <v>-1.2678644005712723e-14</v>
@@ -2013,16 +2019,16 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>0.6202949310831237</v>
+        <v>-0.5851956049269981</v>
       </c>
       <c r="C18">
         <v>0.0</v>
       </c>
       <c r="D18">
-        <v>0.36775375988493847</v>
+        <v>-0.3779051514818019</v>
       </c>
       <c r="E18">
-        <v>0.3961171599492469</v>
+        <v>0.019615529123016506</v>
       </c>
       <c r="F18">
         <v>-1.2267177175878604e-14</v>
@@ -2039,16 +2045,16 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>0.5691926844693418</v>
+        <v>-0.5348503251242684</v>
       </c>
       <c r="C19">
         <v>0.0</v>
       </c>
       <c r="D19">
-        <v>0.35534378731108784</v>
+        <v>-0.36626309791247713</v>
       </c>
       <c r="E19">
-        <v>0.375941241585227</v>
+        <v>0.012295576831416185</v>
       </c>
       <c r="F19">
         <v>-1.1873839922785759e-14</v>
@@ -2065,16 +2071,16 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>0.5202897774842149</v>
+        <v>-0.4865796943485873</v>
       </c>
       <c r="C20">
         <v>0.0</v>
       </c>
       <c r="D20">
-        <v>0.3433055700353413</v>
+        <v>-0.35379549635816077</v>
       </c>
       <c r="E20">
-        <v>0.3574070387942579</v>
+        <v>0.006247266563694634</v>
       </c>
       <c r="F20">
         <v>-1.1499852516027993e-14</v>
@@ -2091,16 +2097,16 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>0.473548341248213</v>
+        <v>-0.4404176585643645</v>
       </c>
       <c r="C21">
         <v>0.0</v>
       </c>
       <c r="D21">
-        <v>0.3310444218815106</v>
+        <v>-0.34031834310639586</v>
       </c>
       <c r="E21">
-        <v>0.33977496936123824</v>
+        <v>0.00132109198404053</v>
       </c>
       <c r="F21">
         <v>-1.1146005906605964e-14</v>
@@ -2117,16 +2123,16 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>0.4289533027672345</v>
+        <v>-0.39641449189423267</v>
       </c>
       <c r="C22">
         <v>0.0</v>
       </c>
       <c r="D22">
-        <v>0.31821371106204765</v>
+        <v>-0.32578948348292586</v>
       </c>
       <c r="E22">
-        <v>0.3225638534647222</v>
+        <v>-0.0026212333665151647</v>
       </c>
       <c r="F22">
         <v>-1.0812716533065178e-14</v>
@@ -2143,16 +2149,16 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>0.3865114381510728</v>
+        <v>-0.35462541134890396</v>
       </c>
       <c r="C23">
         <v>0.0</v>
       </c>
       <c r="D23">
-        <v>0.3046449940301095</v>
+        <v>-0.31026540410425607</v>
       </c>
       <c r="E23">
-        <v>0.3054812462371977</v>
+        <v>-0.0057067365597778365</v>
       </c>
       <c r="F23">
         <v>-1.0500078033443117e-14</v>
@@ -2169,16 +2175,16 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>0.34624309946252885</v>
+        <v>-0.3151019201212323</v>
       </c>
       <c r="C24">
         <v>0.0</v>
       </c>
       <c r="D24">
-        <v>0.2902962371523612</v>
+        <v>-0.2938683385363192</v>
       </c>
       <c r="E24">
-        <v>0.2883715920369886</v>
+        <v>-0.008051371764514897</v>
       </c>
       <c r="F24">
         <v>-1.0207909511547629e-14</v>
@@ -2195,16 +2201,16 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>0.30817343957405235</v>
+        <v>-0.2778857293158672</v>
       </c>
       <c r="C25">
         <v>0.0</v>
       </c>
       <c r="D25">
-        <v>0.2752128316575503</v>
+        <v>-0.2767613519160847</v>
       </c>
       <c r="E25">
-        <v>0.2711769839938415</v>
+        <v>-0.009760368411796552</v>
       </c>
       <c r="F25">
         <v>-9.935800143135421e-15</v>
@@ -2221,16 +2227,16 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>0.2723252291489793</v>
+        <v>-0.24300483263028988</v>
       </c>
       <c r="C26">
         <v>0.0</v>
       </c>
       <c r="D26">
-        <v>0.2594981156297165</v>
+        <v>-0.2591296411091694</v>
       </c>
       <c r="E26">
-        <v>0.25390729921700655</v>
+        <v>-0.010928692249962738</v>
       </c>
       <c r="F26">
         <v>-9.683150018825644e-15</v>
@@ -2247,16 +2253,16 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>0.2387136511414243</v>
+        <v>-0.2104712802923241</v>
       </c>
       <c r="C27">
         <v>0.0</v>
       </c>
       <c r="D27">
-        <v>0.24329115253479333</v>
+        <v>-0.24116668668256175</v>
       </c>
       <c r="E27">
-        <v>0.2366175013392508</v>
+        <v>-0.011641582036532809</v>
       </c>
       <c r="F27">
         <v>-9.449207209792284e-15</v>
@@ -2273,16 +2279,16 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>0.20734289002415335</v>
+        <v>-0.18028024939896087</v>
       </c>
       <c r="C28">
         <v>0.0</v>
       </c>
       <c r="D28">
-        <v>0.22675012020918134</v>
+        <v>-0.22306418926392452</v>
       </c>
       <c r="E28">
-        <v>0.2193904961467077</v>
+        <v>-0.011975133399397053</v>
       </c>
       <c r="F28">
         <v>-9.233101112711743e-15</v>
@@ -2299,16 +2305,16 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>0.17820418491658996</v>
+        <v>-0.15241007639848064</v>
       </c>
       <c r="C29">
         <v>0.0</v>
       </c>
       <c r="D29">
-        <v>0.2100400594585057</v>
+        <v>-0.20500494976223432</v>
       </c>
       <c r="E29">
-        <v>0.20232431352900054</v>
+        <v>-0.011996908170405237</v>
       </c>
       <c r="F29">
         <v>-9.033872184976306e-15</v>
@@ -2325,16 +2331,16 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>0.15127501466405358</v>
+        <v>-0.12682298287541582</v>
       </c>
       <c r="C30">
         <v>0.0</v>
       </c>
       <c r="D30">
-        <v>0.19332401223674595</v>
+        <v>-0.18715802973435192</v>
       </c>
       <c r="E30">
-        <v>0.18552266391158495</v>
+        <v>-0.011766552744396662</v>
       </c>
       <c r="F30">
         <v>-8.850498222334385e-15</v>
@@ -2351,16 +2357,16 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>0.1265191267727281</v>
+        <v>-0.10346628204886194</v>
       </c>
       <c r="C31">
         <v>0.0</v>
       </c>
       <c r="D31">
-        <v>0.1767567894266234</v>
+        <v>-0.16967566721733235</v>
       </c>
       <c r="E31">
-        <v>0.1690881228443292</v>
+        <v>-0.01133641309897367</v>
       </c>
       <c r="F31">
         <v>-8.681917361073525e-15</v>
@@ -2377,16 +2383,16 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>0.10388717416473889</v>
+        <v>-0.0822738998007228</v>
       </c>
       <c r="C32">
         <v>0.0</v>
       </c>
       <c r="D32">
-        <v>0.16048076990975907</v>
+        <v>-0.1526915332110001</v>
       </c>
       <c r="E32">
-        <v>0.15311735557648556</v>
+        <v>-0.010752137288434079</v>
       </c>
       <c r="F32">
         <v>-8.527048007516854e-15</v>
@@ -2403,16 +2409,16 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>0.08331777173485576</v>
+        <v>-0.06316808163341717</v>
       </c>
       <c r="C33">
         <v>0.0</v>
       </c>
       <c r="D33">
-        <v>0.14462325893598377</v>
+        <v>-0.13632000105110623</v>
       </c>
       <c r="E33">
-        <v>0.13769791704712447</v>
+        <v>-0.010053258700306674</v>
       </c>
       <c r="F33">
         <v>-8.384805910596488e-15</v>
@@ -2429,16 +2435,16 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>0.06473882543354056</v>
+        <v>-0.046061187124972265</v>
       </c>
       <c r="C34">
         <v>0.0</v>
       </c>
       <c r="D34">
-        <v>0.12929503328462028</v>
+        <v>-0.12065617001690093</v>
       </c>
       <c r="E34">
-        <v>0.12290626009298944</v>
+        <v>-0.009273755289992894</v>
       </c>
       <c r="F34">
         <v>-8.254118600003628e-15</v>
@@ -2455,16 +2461,16 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>0.04806901999222726</v>
+        <v>-0.03085749755064561</v>
       </c>
       <c r="C35">
         <v>0.0</v>
       </c>
       <c r="D35">
-        <v>0.1145897793898969</v>
+        <v>-0.10577643943910728</v>
       </c>
       <c r="E35">
-        <v>0.10880666171970085</v>
+        <v>-0.008442581508415481</v>
       </c>
       <c r="F35">
         <v>-8.133937414100203e-15</v>
@@ -2481,16 +2487,16 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>0.03321937833689396</v>
+        <v>-0.01745498153316079</v>
       </c>
       <c r="C36">
         <v>0.0</v>
       </c>
       <c r="D36">
-        <v>0.10058419297843774</v>
+        <v>-0.09173947326853786</v>
       </c>
       <c r="E36">
-        <v>0.09545083839271665</v>
+        <v>-0.007584170802837485</v>
       </c>
       <c r="F36">
         <v>-8.023247339437343e-15</v>
@@ -2507,16 +2513,16 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>0.020094827277761112</v>
+        <v>-0.005746978823673742</v>
       </c>
       <c r="C37">
         <v>0.0</v>
       </c>
       <c r="D37">
-        <v>0.08733855829167206</v>
+        <v>-0.07858742985557152</v>
       </c>
       <c r="E37">
-        <v>0.08287806985257444</v>
+        <v>-0.006718907474924289</v>
       </c>
       <c r="F37">
         <v>-7.92107487823219e-15</v>
@@ -2533,16 +2539,16 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>0.00859572120902587</v>
+        <v>0.0043762256228740805</v>
       </c>
       <c r="C38">
         <v>0.0</v>
       </c>
       <c r="D38">
-        <v>0.07489766432802991</v>
+        <v>-0.06634735940908407</v>
       </c>
       <c r="E38">
-        <v>0.07111568956938276</v>
+        <v>-0.0058635673793306885</v>
       </c>
       <c r="F38">
         <v>-7.826494152242911e-15</v>
@@ -2559,16 +2565,16 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>-0.0013807108535275074</v>
+        <v>0.013025955608796925</v>
       </c>
       <c r="C39">
         <v>0.0</v>
       </c>
       <c r="D39">
-        <v>0.06329194684754574</v>
+        <v>-0.05503269369781794</v>
       </c>
       <c r="E39">
-        <v>0.06017983068364183</v>
+        <v>-0.0050317274847183355</v>
       </c>
       <c r="F39">
         <v>-7.738631441769198e-15</v>
@@ -2585,16 +2591,16 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>-0.009939018834928658</v>
+        <v>0.020313836572422195</v>
       </c>
       <c r="C40">
         <v>0.0</v>
       </c>
       <c r="D40">
-        <v>0.05253876979570426</v>
+        <v>-0.04464477017242626</v>
       </c>
       <c r="E40">
-        <v>0.050076340756670765</v>
+        <v>-0.004234144731499447</v>
       </c>
       <c r="F40">
         <v>-7.656668347508482e-15</v>
@@ -2611,16 +2617,16 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>-0.017184301266061693</v>
+        <v>0.026350632471733648</v>
       </c>
       <c r="C41">
         <v>0.0</v>
       </c>
       <c r="D41">
-        <v>0.04264377963499199</v>
+        <v>-0.035174346728825516</v>
       </c>
       <c r="E41">
-        <v>0.040801798155347124</v>
+        <v>-0.003479104933536299</v>
       </c>
       <c r="F41">
         <v>-7.579843751144125e-15</v>

</xml_diff>

<commit_message>
EA estimates updated - Full MCMC still to run but mode is robust! US also re-estimated
</commit_message>
<xml_diff>
--- a/irf/irf/Paper IRFs.xlsx
+++ b/irf/irf/Paper IRFs.xlsx
@@ -17,6 +17,9 @@
     <sheet name="FTPL_Equilibrium_IRF_Policy_rat" r:id="rId5" sheetId="2"/>
     <sheet name="FG_6horizon_policy_rate_output_" r:id="rId7" sheetId="3"/>
     <sheet name="FG_6horizon_shock_weights" r:id="rId8" sheetId="4"/>
+    <sheet name="Interest_rate_peg_IRF_Policy_ra" r:id="rId9" sheetId="5"/>
+    <sheet name="stanadard_interest_rate_peg_wit" r:id="rId10" sheetId="6"/>
+    <sheet name="interest_rate_peg_with_only_FG_" r:id="rId11" sheetId="7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="51">
   <si>
     <t>t</t>
   </si>
@@ -115,6 +118,72 @@
   </si>
   <si>
     <t>2026-02-23T14:36:29.843</t>
+  </si>
+  <si>
+    <t>2026-02-26T12:54:28.153</t>
+  </si>
+  <si>
+    <t>2026-02-26T12:55:03.234</t>
+  </si>
+  <si>
+    <t>2026-02-26T12:55:08.508</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:05:39.525</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:05:56.585</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:06:01.228</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:06:07.945</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:06:10.979</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:06:37.014</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:14:52.476</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:15:57.219</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:16:00.719</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:16:03.9</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:16:06.861</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:16:10.012</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:16:13.832</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:19:49.297</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:19:55.616</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:20:00.281</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:20:04.254</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:20:07.563</t>
+  </si>
+  <si>
+    <t>2026-02-27T23:20:10.748</t>
   </si>
 </sst>
 </file>
@@ -495,16 +564,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
@@ -516,7 +585,7 @@
         <v>8</v>
       </c>
       <c r="K1" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -527,22 +596,22 @@
         <v>-1.0</v>
       </c>
       <c r="C2">
-        <v>-1.6915336844286093</v>
+        <v>0.0</v>
       </c>
       <c r="D2">
-        <v>0.0</v>
+        <v>3.111383456359226e-15</v>
       </c>
       <c r="E2">
-        <v>5.148080382766119e-15</v>
+        <v>0.07166727228172108</v>
       </c>
       <c r="F2">
-        <v>0.0716672722817191</v>
+        <v>-1.69153368442861</v>
       </c>
       <c r="G2">
-        <v>2.5793795815169456</v>
+        <v>2.5793795815169407</v>
       </c>
       <c r="H2">
-        <v>-1.0776287571287195</v>
+        <v>-1.077628757128724</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -553,22 +622,22 @@
         <v>-1.0</v>
       </c>
       <c r="C3">
-        <v>-0.7378682177184183</v>
+        <v>0.0</v>
       </c>
       <c r="D3">
-        <v>0.0</v>
+        <v>3.898465206358163e-15</v>
       </c>
       <c r="E3">
-        <v>6.2791836394635625e-15</v>
+        <v>0.09633801591550874</v>
       </c>
       <c r="F3">
-        <v>0.09633801591550183</v>
+        <v>-0.7378682177184217</v>
       </c>
       <c r="G3">
-        <v>1.4953394328181018</v>
+        <v>1.495339432818104</v>
       </c>
       <c r="H3">
-        <v>-1.0901798523912853</v>
+        <v>-1.0901798523912902</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -579,22 +648,22 @@
         <v>-1.0</v>
       </c>
       <c r="C4">
-        <v>-0.6713986913636436</v>
+        <v>0.0</v>
       </c>
       <c r="D4">
-        <v>0.0</v>
+        <v>4.940492912591414e-15</v>
       </c>
       <c r="E4">
-        <v>7.804041398192428e-15</v>
+        <v>0.11514371513779122</v>
       </c>
       <c r="F4">
-        <v>0.11514371513778257</v>
+        <v>-0.6713986913636477</v>
       </c>
       <c r="G4">
-        <v>1.1447890872423834</v>
+        <v>1.144789087242387</v>
       </c>
       <c r="H4">
-        <v>-1.1050722210876067</v>
+        <v>-1.105072221087612</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -605,22 +674,22 @@
         <v>-1.0</v>
       </c>
       <c r="C5">
-        <v>-0.6279689939410035</v>
+        <v>0.0</v>
       </c>
       <c r="D5">
-        <v>0.0</v>
+        <v>5.93655304045774e-15</v>
       </c>
       <c r="E5">
-        <v>9.213698585158189e-15</v>
+        <v>0.12932449243634242</v>
       </c>
       <c r="F5">
-        <v>0.12932449243633257</v>
+        <v>-0.6279689939410079</v>
       </c>
       <c r="G5">
         <v>0.9056919935333063</v>
       </c>
       <c r="H5">
-        <v>-1.1161558581396847</v>
+        <v>-1.1161558581396904</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -631,22 +700,22 @@
         <v>-1.0</v>
       </c>
       <c r="C6">
-        <v>-0.5973455825607836</v>
+        <v>0.0</v>
       </c>
       <c r="D6">
-        <v>0.0</v>
+        <v>6.895917639831189e-15</v>
       </c>
       <c r="E6">
-        <v>1.0529939632425284e-14</v>
+        <v>0.13989587911805162</v>
       </c>
       <c r="F6">
-        <v>0.1398958791180408</v>
+        <v>-0.5973455825607896</v>
       </c>
       <c r="G6">
-        <v>0.7319914235132261</v>
+        <v>0.7319914235132314</v>
       </c>
       <c r="H6">
-        <v>-1.124275171477677</v>
+        <v>-1.124275171477683</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -657,22 +726,22 @@
         <v>-1.0</v>
       </c>
       <c r="C7">
-        <v>-0.5737467099099121</v>
+        <v>0.0</v>
       </c>
       <c r="D7">
-        <v>0.0</v>
+        <v>7.822472301516801e-15</v>
       </c>
       <c r="E7">
-        <v>1.1764561194408219e-14</v>
+        <v>0.14757978149828713</v>
       </c>
       <c r="F7">
-        <v>0.14757978149827572</v>
+        <v>-0.5737467099099169</v>
       </c>
       <c r="G7">
-        <v>0.5973427245187732</v>
+        <v>0.5973427245187759</v>
       </c>
       <c r="H7">
-        <v>-1.1300125312110396</v>
+        <v>-1.1300125312110456</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -680,25 +749,25 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>-0.7449269414029471</v>
+        <v>-0.7449269414029468</v>
       </c>
       <c r="C8">
-        <v>-0.12249492256576702</v>
+        <v>0.0</v>
       </c>
       <c r="D8">
-        <v>0.0</v>
+        <v>7.92371673135295e-15</v>
       </c>
       <c r="E8">
-        <v>1.1610965451139857e-14</v>
+        <v>0.13461497481591014</v>
       </c>
       <c r="F8">
-        <v>0.13461497481589896</v>
+        <v>-0.12249492256576862</v>
       </c>
       <c r="G8">
         <v>-0.1711148877063895</v>
       </c>
       <c r="H8">
-        <v>-0.8589162460761607</v>
+        <v>-0.8589162460761651</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -706,25 +775,25 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>-0.5546326047314784</v>
+        <v>-0.5546326047314788</v>
       </c>
       <c r="C9">
-        <v>-0.02615266596779151</v>
+        <v>0.0</v>
       </c>
       <c r="D9">
-        <v>0.0</v>
+        <v>7.993945003915494e-15</v>
       </c>
       <c r="E9">
-        <v>1.1431233203186344e-14</v>
+        <v>0.11802452605864389</v>
       </c>
       <c r="F9">
-        <v>0.11802452605863416</v>
+        <v>-0.026152665967792765</v>
       </c>
       <c r="G9">
-        <v>-0.48020139575093257</v>
+        <v>-0.4802013957509361</v>
       </c>
       <c r="H9">
-        <v>-0.6527917857811548</v>
+        <v>-0.652791785781159</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -732,25 +801,25 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>-0.4349253801348609</v>
+        <v>-0.4349253801348624</v>
       </c>
       <c r="C10">
-        <v>-0.005583594184123434</v>
+        <v>0.0</v>
       </c>
       <c r="D10">
-        <v>0.0</v>
+        <v>8.036648733937131e-15</v>
       </c>
       <c r="E10">
-        <v>1.1231008356708664e-14</v>
+        <v>0.1016340160588325</v>
       </c>
       <c r="F10">
-        <v>0.10163401605882434</v>
+        <v>-0.005583594184124898</v>
       </c>
       <c r="G10">
-        <v>-0.5768324684811983</v>
+        <v>-0.5768324684812018</v>
       </c>
       <c r="H10">
-        <v>-0.518379630721563</v>
+        <v>-0.5183796307215672</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -758,25 +827,25 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>-0.36010806827413905</v>
+        <v>-0.36010806827414216</v>
       </c>
       <c r="C11">
-        <v>-0.0011920973583099271</v>
+        <v>0.0</v>
       </c>
       <c r="D11">
-        <v>0.0</v>
+        <v>8.055177528238005e-15</v>
       </c>
       <c r="E11">
-        <v>1.1015381934708258e-14</v>
+        <v>0.08640853105746768</v>
       </c>
       <c r="F11">
-        <v>0.08640853105746107</v>
+        <v>-0.001192097358311618</v>
       </c>
       <c r="G11">
-        <v>-0.5871768624011784</v>
+        <v>-0.5871768624011837</v>
       </c>
       <c r="H11">
-        <v>-0.4302230951401023</v>
+        <v>-0.4302230951401071</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -784,25 +853,25 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>-0.31207784837616204</v>
+        <v>-0.3120778483761672</v>
       </c>
       <c r="C12">
-        <v>-0.0002545127859985</v>
+        <v>0.0</v>
       </c>
       <c r="D12">
-        <v>0.0</v>
+        <v>8.052694231048553e-15</v>
       </c>
       <c r="E12">
-        <v>1.078889283971475e-14</v>
+        <v>0.0725970988170137</v>
       </c>
       <c r="F12">
-        <v>0.07259709881700852</v>
+        <v>-0.0002545127860002641</v>
       </c>
       <c r="G12">
-        <v>-0.5655516135502099</v>
+        <v>-0.565551613550217</v>
       </c>
       <c r="H12">
-        <v>-0.37025101988486603</v>
+        <v>-0.37025101988487197</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -810,25 +879,25 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>-0.2803966295926651</v>
+        <v>-0.28039662959267125</v>
       </c>
       <c r="C13">
-        <v>-5.4338479809878387e-5</v>
+        <v>0.0</v>
       </c>
       <c r="D13">
-        <v>0.0</v>
+        <v>8.03214546479992e-15</v>
       </c>
       <c r="E13">
-        <v>1.0555540114031353e-14</v>
+        <v>0.06023250178010655</v>
       </c>
       <c r="F13">
-        <v>0.060232501780102726</v>
+        <v>-5.4338479811570196e-5</v>
       </c>
       <c r="G13">
-        <v>-0.5334958471292568</v>
+        <v>-0.5334958471292577</v>
       </c>
       <c r="H13">
-        <v>-0.32798101284319414</v>
+        <v>-0.32798101284320025</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -836,25 +905,25 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>-0.2590128761764773</v>
+        <v>-0.25901287617648544</v>
       </c>
       <c r="C14">
-        <v>-1.1601265438559588e-5</v>
+        <v>0.0</v>
       </c>
       <c r="D14">
-        <v>0.0</v>
+        <v>7.996244402227264e-15</v>
       </c>
       <c r="E14">
-        <v>1.0318803898651284e-14</v>
+        <v>0.04926887041759134</v>
       </c>
       <c r="F14">
-        <v>0.04926887041758877</v>
+        <v>-1.1601265440080863e-5</v>
       </c>
       <c r="G14">
-        <v>-0.499029394560659</v>
+        <v>-0.4990293945606652</v>
       </c>
       <c r="H14">
-        <v>-0.29728557226249874</v>
+        <v>-0.29728557226250607</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -862,25 +931,25 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>-0.244202943146743</v>
+        <v>-0.24420294314675212</v>
       </c>
       <c r="C15">
-        <v>-2.47687017037748e-6</v>
+        <v>0.0</v>
       </c>
       <c r="D15">
-        <v>0.0</v>
+        <v>7.947463158533916e-15</v>
       </c>
       <c r="E15">
-        <v>1.0081672752685055e-14</v>
+        <v>0.03962754952745947</v>
       </c>
       <c r="F15">
-        <v>0.039627549527458145</v>
+        <v>-2.476870171681697e-6</v>
       </c>
       <c r="G15">
-        <v>-0.46490712897908937</v>
+        <v>-0.46490712897909026</v>
       </c>
       <c r="H15">
-        <v>-0.27435118561052385</v>
+        <v>-0.2743511856105313</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -888,25 +957,25 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>-0.2335344033664392</v>
+        <v>-0.2335344033664497</v>
       </c>
       <c r="C16">
-        <v>-5.288117807193205e-7</v>
+        <v>0.0</v>
       </c>
       <c r="D16">
-        <v>0.0</v>
+        <v>7.888032605038842e-15</v>
       </c>
       <c r="E16">
-        <v>9.84667539576941e-15</v>
+        <v>0.031215490246990683</v>
       </c>
       <c r="F16">
-        <v>0.031215490246990597</v>
+        <v>-5.288117817913485e-7</v>
       </c>
       <c r="G16">
-        <v>-0.43193786324030503</v>
+        <v>-0.4319378632403077</v>
       </c>
       <c r="H16">
-        <v>-0.2566500422596416</v>
+        <v>-0.25665004225964966</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -914,25 +983,25 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>-0.22535571436970298</v>
+        <v>-0.22535571436971474</v>
       </c>
       <c r="C17">
-        <v>-1.1290131462664847e-7</v>
+        <v>0.0</v>
       </c>
       <c r="D17">
-        <v>0.0</v>
+        <v>7.819947773804995e-15</v>
       </c>
       <c r="E17">
-        <v>9.615915282630472e-15</v>
+        <v>0.023933932510013023</v>
       </c>
       <c r="F17">
-        <v>0.02393393251001406</v>
+        <v>-1.1290131546558792e-7</v>
       </c>
       <c r="G17">
-        <v>-0.4002656212734461</v>
+        <v>-0.4002656212734492</v>
       </c>
       <c r="H17">
-        <v>-0.24243423152081073</v>
+        <v>-0.24243423152081936</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -940,25 +1009,25 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>-0.21852925238737592</v>
+        <v>-0.2185292523873888</v>
       </c>
       <c r="C18">
-        <v>-2.4104430213144082e-8</v>
+        <v>0.0</v>
       </c>
       <c r="D18">
-        <v>0.0</v>
+        <v>7.744977345828397e-15</v>
       </c>
       <c r="E18">
-        <v>9.391106717500153e-15</v>
+        <v>0.017683096658247664</v>
       </c>
       <c r="F18">
-        <v>0.017683096658249697</v>
+        <v>-2.41044308264451e-8</v>
       </c>
       <c r="G18">
-        <v>-0.3698442820958281</v>
+        <v>-0.36984428209583076</v>
       </c>
       <c r="H18">
-        <v>-0.23047147775076154</v>
+        <v>-0.23047147775077065</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -966,25 +1035,25 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>-0.21227671283745408</v>
+        <v>-0.2122767128374673</v>
       </c>
       <c r="C19">
-        <v>-5.146295484060616e-9</v>
+        <v>0.0</v>
       </c>
       <c r="D19">
-        <v>0.0</v>
+        <v>7.664675995318849e-15</v>
       </c>
       <c r="E19">
-        <v>9.173611471779076e-15</v>
+        <v>0.012364980141239663</v>
       </c>
       <c r="F19">
-        <v>0.012364980141242678</v>
+        <v>-5.14629588454877e-9</v>
       </c>
       <c r="G19">
-        <v>-0.34060187362750494</v>
+        <v>-0.34060187362750627</v>
       </c>
       <c r="H19">
-        <v>-0.2198922430955447</v>
+        <v>-0.21989224309555344</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -992,25 +1061,25 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>-0.2060797172707384</v>
+        <v>-0.2060797172707516</v>
       </c>
       <c r="C20">
-        <v>-1.098733807066088e-9</v>
+        <v>0.0</v>
       </c>
       <c r="D20">
-        <v>0.0</v>
+        <v>7.580398602510176e-15</v>
       </c>
       <c r="E20">
-        <v>8.964475086133216e-15</v>
+        <v>0.007885120029216744</v>
       </c>
       <c r="F20">
-        <v>0.007885120029220665</v>
+        <v>-1.0987340110261482e-9</v>
       </c>
       <c r="G20">
-        <v>-0.31248901919794614</v>
+        <v>-0.3124890191979479</v>
       </c>
       <c r="H20">
-        <v>-0.21009142183175822</v>
+        <v>-0.21009142183176638</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -1018,25 +1087,25 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>-0.19961054127213992</v>
+        <v>-0.19961054127215333</v>
       </c>
       <c r="C21">
-        <v>-2.34579470172812e-10</v>
+        <v>0.0</v>
       </c>
       <c r="D21">
-        <v>0.0</v>
+        <v>7.49331555098882e-15</v>
       </c>
       <c r="E21">
-        <v>8.76446222262879e-15</v>
+        <v>0.0041537189024692745</v>
       </c>
       <c r="F21">
-        <v>0.004153718902474034</v>
+        <v>-2.345794959814191e-10</v>
       </c>
       <c r="G21">
-        <v>-0.2854862761513888</v>
+        <v>-0.28548627615138966</v>
       </c>
       <c r="H21">
-        <v>-0.20065974270055495</v>
+        <v>-0.20065974270056278</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -1592,13 +1661,13 @@
         <v>8</v>
       </c>
       <c r="H1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="J1" t="s">
         <v>8</v>
       </c>
       <c r="K1" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -1606,25 +1675,25 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>8.102500031716193</v>
+        <v>8.102500031716206</v>
       </c>
       <c r="C2">
         <v>0.0</v>
       </c>
       <c r="D2">
-        <v>-1.0</v>
+        <v>-0.9999999999999997</v>
       </c>
       <c r="E2">
-        <v>0.3002694365653483</v>
+        <v>0.30026943656535576</v>
       </c>
       <c r="F2">
-        <v>-1.8240941779797443e-14</v>
+        <v>1.1945048918812522e-14</v>
       </c>
       <c r="G2">
-        <v>0.4586028719414255</v>
+        <v>-3.200818256209439</v>
       </c>
       <c r="H2">
-        <v>-0.2916108571679106</v>
+        <v>0.30026943656535576</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1632,25 +1701,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3.7924900644128168</v>
+        <v>11.894990096129039</v>
       </c>
       <c r="C3">
         <v>0.0</v>
       </c>
       <c r="D3">
-        <v>-1.0</v>
+        <v>-0.9999999999999998</v>
       </c>
       <c r="E3">
-        <v>0.34132427283477856</v>
+        <v>0.341324272834796</v>
       </c>
       <c r="F3">
-        <v>-1.815767595640473e-14</v>
+        <v>1.236786245210933e-14</v>
       </c>
       <c r="G3">
-        <v>0.22319313455430967</v>
+        <v>-0.8007358613175596</v>
       </c>
       <c r="H3">
-        <v>-0.33915754479465826</v>
+        <v>0.341324272834796</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1658,25 +1727,25 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1.535682253088882</v>
+        <v>13.430672349217918</v>
       </c>
       <c r="C4">
         <v>0.0</v>
       </c>
       <c r="D4">
-        <v>-1.0000000000000002</v>
+        <v>-0.9999999999999999</v>
       </c>
       <c r="E4">
-        <v>0.3262395395059982</v>
+        <v>0.3262395395060162</v>
       </c>
       <c r="F4">
-        <v>-1.7990016981340348e-14</v>
+        <v>1.2712130219558677e-14</v>
       </c>
       <c r="G4">
-        <v>0.1733771867033961</v>
+        <v>-0.6225725146161963</v>
       </c>
       <c r="H4">
-        <v>-0.3359955377002835</v>
+        <v>0.3262395395060162</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1684,25 +1753,25 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.314417515476746</v>
+        <v>13.74508986469466</v>
       </c>
       <c r="C5">
         <v>0.0</v>
       </c>
       <c r="D5">
-        <v>-1.0</v>
+        <v>-0.9999999999999998</v>
       </c>
       <c r="E5">
-        <v>0.297172637639562</v>
+        <v>0.29717263763957846</v>
       </c>
       <c r="F5">
-        <v>-1.7750026373046594e-14</v>
+        <v>1.2984205210219286e-14</v>
       </c>
       <c r="G5">
-        <v>0.13606624062531894</v>
+        <v>-0.4304117562920385</v>
       </c>
       <c r="H5">
-        <v>-0.3194967604267872</v>
+        <v>0.29717263763957846</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1710,25 +1779,25 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>-0.3714566512920629</v>
+        <v>13.373633213402588</v>
       </c>
       <c r="C6">
         <v>0.0</v>
       </c>
       <c r="D6">
-        <v>-1.0000000000000002</v>
+        <v>-1.0</v>
       </c>
       <c r="E6">
-        <v>0.26450237048056346</v>
+        <v>0.26450237048057795</v>
       </c>
       <c r="F6">
-        <v>-1.7449311279723872e-14</v>
+        <v>1.3190713735165675e-14</v>
       </c>
       <c r="G6">
-        <v>0.10077323633482921</v>
+        <v>-0.3107196037060323</v>
       </c>
       <c r="H6">
-        <v>-0.2975542049811292</v>
+        <v>0.26450237048057795</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1736,25 +1805,25 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>-0.7682647916323465</v>
+        <v>12.605368421770233</v>
       </c>
       <c r="C7">
         <v>0.0</v>
       </c>
       <c r="D7">
-        <v>-1.0</v>
+        <v>-0.9999999999999999</v>
       </c>
       <c r="E7">
-        <v>0.23168373759607122</v>
+        <v>0.23168373759608402</v>
       </c>
       <c r="F7">
-        <v>-1.7098845668544484e-14</v>
+        <v>1.3338330603505361e-14</v>
       </c>
       <c r="G7">
-        <v>2.063782970431286</v>
+        <v>-0.231532170537758</v>
       </c>
       <c r="H7">
-        <v>-0.27236297336873977</v>
+        <v>0.23168373759608402</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1762,25 +1831,25 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>-0.9983762771240359</v>
+        <v>11.60699214464619</v>
       </c>
       <c r="C8">
         <v>0.0</v>
       </c>
       <c r="D8">
-        <v>-0.8228559440075205</v>
+        <v>-0.8228559440075245</v>
       </c>
       <c r="E8">
-        <v>0.20029060488665273</v>
+        <v>0.20029060488666367</v>
       </c>
       <c r="F8">
-        <v>-1.6708846025861055e-14</v>
+        <v>1.3433608185646603e-14</v>
       </c>
       <c r="G8">
         <v>0.0</v>
       </c>
       <c r="H8">
-        <v>-0.2449613808818707</v>
+        <v>0.20029060488666367</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1788,25 +1857,25 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>-1.0615234494165005</v>
+        <v>10.545468695229683</v>
       </c>
       <c r="C9">
         <v>0.0</v>
       </c>
       <c r="D9">
-        <v>-0.6802281125838083</v>
+        <v>-0.6802281125838165</v>
       </c>
       <c r="E9">
-        <v>0.17117303992476582</v>
+        <v>0.17117303992477478</v>
       </c>
       <c r="F9">
-        <v>-1.628869161461582e-14</v>
+        <v>1.3482850291698822e-14</v>
       </c>
       <c r="G9">
         <v>0.0</v>
       </c>
       <c r="H9">
-        <v>-0.21613136847009748</v>
+        <v>0.17117303992477478</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1814,25 +1883,25 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>-1.0428589933721009</v>
+        <v>9.502609701857576</v>
       </c>
       <c r="C10">
         <v>0.0</v>
       </c>
       <c r="D10">
-        <v>-0.5839658177105793</v>
+        <v>-0.5839658177105909</v>
       </c>
       <c r="E10">
-        <v>0.14469354968982942</v>
+        <v>0.1446935496898365</v>
       </c>
       <c r="F10">
-        <v>-1.5846880766101665e-14</v>
+        <v>1.3492022862886328e-14</v>
       </c>
       <c r="G10">
         <v>0.0</v>
       </c>
       <c r="H10">
-        <v>-0.18772319729264852</v>
+        <v>0.1446935496898365</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1840,25 +1909,25 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>-0.9921377386601233</v>
+        <v>8.51047196319744</v>
       </c>
       <c r="C11">
         <v>0.0</v>
       </c>
       <c r="D11">
-        <v>-0.5204572812941362</v>
+        <v>-0.5204572812941508</v>
       </c>
       <c r="E11">
-        <v>0.1209314480216968</v>
+        <v>0.12093144802170196</v>
       </c>
       <c r="F11">
-        <v>-1.5391015939674246e-14</v>
+        <v>1.3466694517385076e-14</v>
       </c>
       <c r="G11">
         <v>0.0</v>
       </c>
       <c r="H11">
-        <v>-0.16101066831640803</v>
+        <v>0.12093144802170196</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1866,25 +1935,25 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>-0.9313171317033377</v>
+        <v>7.579154831494095</v>
       </c>
       <c r="C12">
         <v>0.0</v>
       </c>
       <c r="D12">
-        <v>-0.4780823352039272</v>
+        <v>-0.4780823352039434</v>
       </c>
       <c r="E12">
-        <v>0.0998197529172179</v>
+        <v>0.0998197529172211</v>
       </c>
       <c r="F12">
-        <v>-1.492781138475873e-14</v>
+        <v>1.3412000973304146e-14</v>
       </c>
       <c r="G12">
         <v>0.0</v>
       </c>
       <c r="H12">
-        <v>-0.13659061073591336</v>
+        <v>0.0998197529172211</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1892,25 +1961,25 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>-0.8688979012157303</v>
+        <v>6.710256930278353</v>
       </c>
       <c r="C13">
         <v>0.0</v>
       </c>
       <c r="D13">
-        <v>-0.44914320705740507</v>
+        <v>-0.4491432070574239</v>
       </c>
       <c r="E13">
-        <v>0.08122018743975548</v>
+        <v>0.08122018743975679</v>
       </c>
       <c r="F13">
-        <v>-1.4463118201713377e-14</v>
+        <v>1.3332628271158423e-14</v>
       </c>
       <c r="G13">
         <v>0.0</v>
       </c>
       <c r="H13">
-        <v>-0.11464720511777625</v>
+        <v>0.08122018743975679</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1918,25 +1987,25 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>-0.8077995380727517</v>
+        <v>5.9024573922055925</v>
       </c>
       <c r="C14">
         <v>0.0</v>
       </c>
       <c r="D14">
-        <v>-0.42862347099199605</v>
+        <v>-0.42862347099201664</v>
       </c>
       <c r="E14">
-        <v>0.06496131838760792</v>
+        <v>0.06496131838760731</v>
       </c>
       <c r="F14">
-        <v>-1.4001962437076097e-14</v>
+        <v>1.323281052728338e-14</v>
       </c>
       <c r="G14">
         <v>0.0</v>
       </c>
       <c r="H14">
-        <v>-0.09515749882355357</v>
+        <v>0.06496131838760731</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1944,25 +2013,25 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>-0.7488403124163857</v>
+        <v>5.153617079789201</v>
       </c>
       <c r="C15">
         <v>0.0</v>
       </c>
       <c r="D15">
-        <v>-0.41317369462819337</v>
+        <v>-0.4131736946282153</v>
       </c>
       <c r="E15">
-        <v>0.05085802283127187</v>
+        <v>0.05085802283126942</v>
       </c>
       <c r="F15">
-        <v>-1.3548592577989773e-14</v>
+        <v>1.3116338666312405e-14</v>
       </c>
       <c r="G15">
         <v>0.0</v>
       </c>
       <c r="H15">
-        <v>-0.07800296479349081</v>
+        <v>0.05085802283126942</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1970,25 +2039,25 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>-0.6921339810602081</v>
+        <v>4.461483098728982</v>
       </c>
       <c r="C16">
         <v>0.0</v>
       </c>
       <c r="D16">
-        <v>-0.4005166921982795</v>
+        <v>-0.40051669219830294</v>
       </c>
       <c r="E16">
-        <v>0.03872194353595661</v>
+        <v>0.038721943535952465</v>
       </c>
       <c r="F16">
-        <v>-1.3106533442287815e-14</v>
+        <v>1.2986577207574162e-14</v>
       </c>
       <c r="G16">
         <v>0.0</v>
       </c>
       <c r="H16">
-        <v>-0.0630235728390008</v>
+        <v>0.038721943535952465</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1996,25 +2065,25 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>-0.6376112097334082</v>
+        <v>3.8238718889955634</v>
       </c>
       <c r="C17">
         <v>0.0</v>
       </c>
       <c r="D17">
-        <v>-0.38910425750694966</v>
+        <v>-0.38910425750697364</v>
       </c>
       <c r="E17">
-        <v>0.028367498022029917</v>
+        <v>0.028367498022024082</v>
       </c>
       <c r="F17">
-        <v>-1.2678644005712723e-14</v>
+        <v>1.2846486722289322e-14</v>
       </c>
       <c r="G17">
         <v>0.0</v>
       </c>
       <c r="H17">
-        <v>-0.050043438695366003</v>
+        <v>0.028367498022024082</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2022,25 +2091,25 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>-0.5851956049269981</v>
+        <v>3.238676284068557</v>
       </c>
       <c r="C18">
         <v>0.0</v>
       </c>
       <c r="D18">
-        <v>-0.3779051514818019</v>
+        <v>-0.37790515148182624</v>
       </c>
       <c r="E18">
-        <v>0.019615529123016506</v>
+        <v>0.01961552912300906</v>
       </c>
       <c r="F18">
-        <v>-1.2267177175878604e-14</v>
+        <v>1.2698650042513726e-14</v>
       </c>
       <c r="G18">
         <v>0.0</v>
       </c>
       <c r="H18">
-        <v>-0.038883382573900116</v>
+        <v>0.01961552912300906</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2048,25 +2117,25 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>-0.5348503251242684</v>
+        <v>2.703825958944279</v>
       </c>
       <c r="C19">
         <v>0.0</v>
       </c>
       <c r="D19">
-        <v>-0.36626309791247713</v>
+        <v>-0.3662630979125017</v>
       </c>
       <c r="E19">
-        <v>0.012295576831416185</v>
+        <v>0.012295576831407232</v>
       </c>
       <c r="F19">
-        <v>-1.1873839922785759e-14</v>
+        <v>1.2545300696393843e-14</v>
       </c>
       <c r="G19">
         <v>0.0</v>
       </c>
       <c r="H19">
-        <v>-0.029367464426574542</v>
+        <v>0.012295576831407232</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2074,25 +2143,25 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>-0.4865796943485873</v>
+        <v>2.217246264595686</v>
       </c>
       <c r="C20">
         <v>0.0</v>
       </c>
       <c r="D20">
-        <v>-0.35379549635816077</v>
+        <v>-0.35379549635818497</v>
       </c>
       <c r="E20">
-        <v>0.006247266563694634</v>
+        <v>0.00624726656368428</v>
       </c>
       <c r="F20">
-        <v>-1.1499852516027993e-14</v>
+        <v>1.2388352375174012e-14</v>
       </c>
       <c r="G20">
         <v>0.0</v>
       </c>
       <c r="H20">
-        <v>-0.021326604155434102</v>
+        <v>0.00624726656368428</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2100,25 +2169,25 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>-0.4404176585643645</v>
+        <v>1.7768286060313154</v>
       </c>
       <c r="C21">
         <v>0.0</v>
       </c>
       <c r="D21">
-        <v>-0.34031834310639586</v>
+        <v>-0.3403183431064198</v>
       </c>
       <c r="E21">
-        <v>0.00132109198404053</v>
+        <v>0.0013210919840288618</v>
       </c>
       <c r="F21">
-        <v>-1.1146005906605964e-14</v>
+        <v>1.2229428513066768e-14</v>
       </c>
       <c r="G21">
         <v>0.0</v>
       </c>
       <c r="H21">
-        <v>-0.014600660752973445</v>
+        <v>0.0013210919840288618</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2665,7 +2734,7 @@
         <v>8</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2673,7 +2742,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>-3.2008182562094296</v>
+        <v>-3.200818256209439</v>
       </c>
       <c r="C2">
         <v>0.0</v>
@@ -2684,7 +2753,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>-0.8007358613175475</v>
+        <v>-0.8007358613175596</v>
       </c>
       <c r="C3">
         <v>0.0</v>
@@ -2695,7 +2764,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>-0.6225725146161908</v>
+        <v>-0.6225725146161963</v>
       </c>
       <c r="C4">
         <v>0.0</v>
@@ -2706,7 +2775,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>-0.43041175629203515</v>
+        <v>-0.4304117562920385</v>
       </c>
       <c r="C5">
         <v>0.0</v>
@@ -2717,7 +2786,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>-0.31071960370603274</v>
+        <v>-0.3107196037060323</v>
       </c>
       <c r="C6">
         <v>0.0</v>
@@ -2728,7 +2797,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>-0.2315321705377608</v>
+        <v>-0.231532170537758</v>
       </c>
       <c r="C7">
         <v>0.0</v>
@@ -3106,6 +3175,1692 @@
       </c>
       <c r="C41">
         <v>0.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
+  <dimension ref="A1:K21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>-1.0</v>
+      </c>
+      <c r="C2">
+        <v>-1.69153368442861</v>
+      </c>
+      <c r="D2">
+        <v>0.0</v>
+      </c>
+      <c r="E2">
+        <v>3.111383456359226e-15</v>
+      </c>
+      <c r="F2">
+        <v>0.07166727228172108</v>
+      </c>
+      <c r="G2">
+        <v>2.5793795815169407</v>
+      </c>
+      <c r="H2">
+        <v>-1.077628757128724</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>-1.0</v>
+      </c>
+      <c r="C3">
+        <v>-0.7378682177184217</v>
+      </c>
+      <c r="D3">
+        <v>0.0</v>
+      </c>
+      <c r="E3">
+        <v>3.898465206358163e-15</v>
+      </c>
+      <c r="F3">
+        <v>0.09633801591550874</v>
+      </c>
+      <c r="G3">
+        <v>1.495339432818104</v>
+      </c>
+      <c r="H3">
+        <v>-1.0901798523912902</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>-1.0</v>
+      </c>
+      <c r="C4">
+        <v>-0.6713986913636477</v>
+      </c>
+      <c r="D4">
+        <v>0.0</v>
+      </c>
+      <c r="E4">
+        <v>4.940492912591414e-15</v>
+      </c>
+      <c r="F4">
+        <v>0.11514371513779122</v>
+      </c>
+      <c r="G4">
+        <v>1.144789087242387</v>
+      </c>
+      <c r="H4">
+        <v>-1.105072221087612</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>-1.0</v>
+      </c>
+      <c r="C5">
+        <v>-0.6279689939410079</v>
+      </c>
+      <c r="D5">
+        <v>0.0</v>
+      </c>
+      <c r="E5">
+        <v>5.93655304045774e-15</v>
+      </c>
+      <c r="F5">
+        <v>0.12932449243634242</v>
+      </c>
+      <c r="G5">
+        <v>0.9056919935333063</v>
+      </c>
+      <c r="H5">
+        <v>-1.1161558581396904</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>-1.0</v>
+      </c>
+      <c r="C6">
+        <v>-0.5973455825607896</v>
+      </c>
+      <c r="D6">
+        <v>0.0</v>
+      </c>
+      <c r="E6">
+        <v>6.895917639831189e-15</v>
+      </c>
+      <c r="F6">
+        <v>0.13989587911805162</v>
+      </c>
+      <c r="G6">
+        <v>0.7319914235132314</v>
+      </c>
+      <c r="H6">
+        <v>-1.124275171477683</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>-1.0</v>
+      </c>
+      <c r="C7">
+        <v>-0.5737467099099169</v>
+      </c>
+      <c r="D7">
+        <v>0.0</v>
+      </c>
+      <c r="E7">
+        <v>7.822472301516801e-15</v>
+      </c>
+      <c r="F7">
+        <v>0.14757978149828713</v>
+      </c>
+      <c r="G7">
+        <v>0.5973427245187759</v>
+      </c>
+      <c r="H7">
+        <v>-1.1300125312110456</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>-0.7449269414029468</v>
+      </c>
+      <c r="C8">
+        <v>-0.12249492256576862</v>
+      </c>
+      <c r="D8">
+        <v>0.0</v>
+      </c>
+      <c r="E8">
+        <v>7.92371673135295e-15</v>
+      </c>
+      <c r="F8">
+        <v>0.13461497481591014</v>
+      </c>
+      <c r="G8">
+        <v>-0.1711148877063895</v>
+      </c>
+      <c r="H8">
+        <v>-0.8589162460761651</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>-0.5546326047314788</v>
+      </c>
+      <c r="C9">
+        <v>-0.026152665967792765</v>
+      </c>
+      <c r="D9">
+        <v>0.0</v>
+      </c>
+      <c r="E9">
+        <v>7.993945003915494e-15</v>
+      </c>
+      <c r="F9">
+        <v>0.11802452605864389</v>
+      </c>
+      <c r="G9">
+        <v>-0.4802013957509361</v>
+      </c>
+      <c r="H9">
+        <v>-0.652791785781159</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>-0.4349253801348624</v>
+      </c>
+      <c r="C10">
+        <v>-0.005583594184124898</v>
+      </c>
+      <c r="D10">
+        <v>0.0</v>
+      </c>
+      <c r="E10">
+        <v>8.036648733937131e-15</v>
+      </c>
+      <c r="F10">
+        <v>0.1016340160588325</v>
+      </c>
+      <c r="G10">
+        <v>-0.5768324684812018</v>
+      </c>
+      <c r="H10">
+        <v>-0.5183796307215672</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>-0.36010806827414216</v>
+      </c>
+      <c r="C11">
+        <v>-0.001192097358311618</v>
+      </c>
+      <c r="D11">
+        <v>0.0</v>
+      </c>
+      <c r="E11">
+        <v>8.055177528238005e-15</v>
+      </c>
+      <c r="F11">
+        <v>0.08640853105746768</v>
+      </c>
+      <c r="G11">
+        <v>-0.5871768624011837</v>
+      </c>
+      <c r="H11">
+        <v>-0.4302230951401071</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>-0.3120778483761672</v>
+      </c>
+      <c r="C12">
+        <v>-0.0002545127860002641</v>
+      </c>
+      <c r="D12">
+        <v>0.0</v>
+      </c>
+      <c r="E12">
+        <v>8.052694231048553e-15</v>
+      </c>
+      <c r="F12">
+        <v>0.0725970988170137</v>
+      </c>
+      <c r="G12">
+        <v>-0.565551613550217</v>
+      </c>
+      <c r="H12">
+        <v>-0.37025101988487197</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>-0.28039662959267125</v>
+      </c>
+      <c r="C13">
+        <v>-5.4338479811570196e-5</v>
+      </c>
+      <c r="D13">
+        <v>0.0</v>
+      </c>
+      <c r="E13">
+        <v>8.03214546479992e-15</v>
+      </c>
+      <c r="F13">
+        <v>0.06023250178010655</v>
+      </c>
+      <c r="G13">
+        <v>-0.5334958471292577</v>
+      </c>
+      <c r="H13">
+        <v>-0.32798101284320025</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>-0.25901287617648544</v>
+      </c>
+      <c r="C14">
+        <v>-1.1601265440080863e-5</v>
+      </c>
+      <c r="D14">
+        <v>0.0</v>
+      </c>
+      <c r="E14">
+        <v>7.996244402227264e-15</v>
+      </c>
+      <c r="F14">
+        <v>0.04926887041759134</v>
+      </c>
+      <c r="G14">
+        <v>-0.4990293945606652</v>
+      </c>
+      <c r="H14">
+        <v>-0.29728557226250607</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>-0.24420294314675212</v>
+      </c>
+      <c r="C15">
+        <v>-2.476870171681697e-6</v>
+      </c>
+      <c r="D15">
+        <v>0.0</v>
+      </c>
+      <c r="E15">
+        <v>7.947463158533916e-15</v>
+      </c>
+      <c r="F15">
+        <v>0.03962754952745947</v>
+      </c>
+      <c r="G15">
+        <v>-0.46490712897909026</v>
+      </c>
+      <c r="H15">
+        <v>-0.2743511856105313</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>-0.2335344033664497</v>
+      </c>
+      <c r="C16">
+        <v>-5.288117817913485e-7</v>
+      </c>
+      <c r="D16">
+        <v>0.0</v>
+      </c>
+      <c r="E16">
+        <v>7.888032605038842e-15</v>
+      </c>
+      <c r="F16">
+        <v>0.031215490246990683</v>
+      </c>
+      <c r="G16">
+        <v>-0.4319378632403077</v>
+      </c>
+      <c r="H16">
+        <v>-0.25665004225964966</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>-0.22535571436971474</v>
+      </c>
+      <c r="C17">
+        <v>-1.1290131546558792e-7</v>
+      </c>
+      <c r="D17">
+        <v>0.0</v>
+      </c>
+      <c r="E17">
+        <v>7.819947773804995e-15</v>
+      </c>
+      <c r="F17">
+        <v>0.023933932510013023</v>
+      </c>
+      <c r="G17">
+        <v>-0.4002656212734492</v>
+      </c>
+      <c r="H17">
+        <v>-0.24243423152081936</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>-0.2185292523873888</v>
+      </c>
+      <c r="C18">
+        <v>-2.41044308264451e-8</v>
+      </c>
+      <c r="D18">
+        <v>0.0</v>
+      </c>
+      <c r="E18">
+        <v>7.744977345828397e-15</v>
+      </c>
+      <c r="F18">
+        <v>0.017683096658247664</v>
+      </c>
+      <c r="G18">
+        <v>-0.36984428209583076</v>
+      </c>
+      <c r="H18">
+        <v>-0.23047147775077065</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>-0.2122767128374673</v>
+      </c>
+      <c r="C19">
+        <v>-5.14629588454877e-9</v>
+      </c>
+      <c r="D19">
+        <v>0.0</v>
+      </c>
+      <c r="E19">
+        <v>7.664675995318849e-15</v>
+      </c>
+      <c r="F19">
+        <v>0.012364980141239663</v>
+      </c>
+      <c r="G19">
+        <v>-0.34060187362750627</v>
+      </c>
+      <c r="H19">
+        <v>-0.21989224309555344</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>-0.2060797172707516</v>
+      </c>
+      <c r="C20">
+        <v>-1.0987340110261482e-9</v>
+      </c>
+      <c r="D20">
+        <v>0.0</v>
+      </c>
+      <c r="E20">
+        <v>7.580398602510176e-15</v>
+      </c>
+      <c r="F20">
+        <v>0.007885120029216744</v>
+      </c>
+      <c r="G20">
+        <v>-0.3124890191979479</v>
+      </c>
+      <c r="H20">
+        <v>-0.21009142183176638</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>-0.19961054127215333</v>
+      </c>
+      <c r="C21">
+        <v>-2.345794959814191e-10</v>
+      </c>
+      <c r="D21">
+        <v>0.0</v>
+      </c>
+      <c r="E21">
+        <v>7.49331555098882e-15</v>
+      </c>
+      <c r="F21">
+        <v>0.0041537189024692745</v>
+      </c>
+      <c r="G21">
+        <v>-0.28548627615138966</v>
+      </c>
+      <c r="H21">
+        <v>-0.20065974270056278</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
+  <dimension ref="A1:K21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>8.102500031716207</v>
+      </c>
+      <c r="C2">
+        <v>0.0</v>
+      </c>
+      <c r="D2">
+        <v>-0.9999999999999997</v>
+      </c>
+      <c r="E2">
+        <v>-1.329654503413945</v>
+      </c>
+      <c r="F2">
+        <v>1.1945048918812522e-14</v>
+      </c>
+      <c r="G2">
+        <v>-3.200818256209439</v>
+      </c>
+      <c r="H2">
+        <v>0.30026943656535576</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3.792490064412832</v>
+      </c>
+      <c r="C3">
+        <v>0.0</v>
+      </c>
+      <c r="D3">
+        <v>-0.9999999999999998</v>
+      </c>
+      <c r="E3">
+        <v>-1.315085512368188</v>
+      </c>
+      <c r="F3">
+        <v>1.236786245210933e-14</v>
+      </c>
+      <c r="G3">
+        <v>-0.8007358613175596</v>
+      </c>
+      <c r="H3">
+        <v>0.341324272834796</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1.5356822530888818</v>
+      </c>
+      <c r="C4">
+        <v>0.0</v>
+      </c>
+      <c r="D4">
+        <v>-0.9999999999999999</v>
+      </c>
+      <c r="E4">
+        <v>-1.2870123987247313</v>
+      </c>
+      <c r="F4">
+        <v>1.2712130219558677e-14</v>
+      </c>
+      <c r="G4">
+        <v>-0.6225725146161963</v>
+      </c>
+      <c r="H4">
+        <v>0.3262395395060162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>0.31441751547674085</v>
+      </c>
+      <c r="C5">
+        <v>0.0</v>
+      </c>
+      <c r="D5">
+        <v>-0.9999999999999998</v>
+      </c>
+      <c r="E5">
+        <v>-1.2554591177135284</v>
+      </c>
+      <c r="F5">
+        <v>1.2984205210219286e-14</v>
+      </c>
+      <c r="G5">
+        <v>-0.4304117562920385</v>
+      </c>
+      <c r="H5">
+        <v>0.29717263763957846</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>-0.37145665129207356</v>
+      </c>
+      <c r="C6">
+        <v>0.0</v>
+      </c>
+      <c r="D6">
+        <v>-1.0</v>
+      </c>
+      <c r="E6">
+        <v>-1.2237625435542734</v>
+      </c>
+      <c r="F6">
+        <v>1.3190713735165675e-14</v>
+      </c>
+      <c r="G6">
+        <v>-0.3107196037060323</v>
+      </c>
+      <c r="H6">
+        <v>0.26450237048057795</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>-0.7682647916323522</v>
+      </c>
+      <c r="C7">
+        <v>0.0</v>
+      </c>
+      <c r="D7">
+        <v>-0.9999999999999999</v>
+      </c>
+      <c r="E7">
+        <v>-1.1934427321679302</v>
+      </c>
+      <c r="F7">
+        <v>1.3338330603505361e-14</v>
+      </c>
+      <c r="G7">
+        <v>-0.231532170537758</v>
+      </c>
+      <c r="H7">
+        <v>0.23168373759608402</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>-0.9983762771240431</v>
+      </c>
+      <c r="C8">
+        <v>0.0</v>
+      </c>
+      <c r="D8">
+        <v>-0.8228559440075245</v>
+      </c>
+      <c r="E8">
+        <v>-0.9881766315918266</v>
+      </c>
+      <c r="F8">
+        <v>1.3433608185646603e-14</v>
+      </c>
+      <c r="G8">
+        <v>0.0</v>
+      </c>
+      <c r="H8">
+        <v>0.20029060488666367</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>-1.0615234494165058</v>
+      </c>
+      <c r="C9">
+        <v>0.0</v>
+      </c>
+      <c r="D9">
+        <v>-0.6802281125838165</v>
+      </c>
+      <c r="E9">
+        <v>-0.8199746353671349</v>
+      </c>
+      <c r="F9">
+        <v>1.3482850291698822e-14</v>
+      </c>
+      <c r="G9">
+        <v>0.0</v>
+      </c>
+      <c r="H9">
+        <v>0.17117303992477478</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>-1.0428589933721049</v>
+      </c>
+      <c r="C10">
+        <v>0.0</v>
+      </c>
+      <c r="D10">
+        <v>-0.5839658177105909</v>
+      </c>
+      <c r="E10">
+        <v>-0.7007626576002115</v>
+      </c>
+      <c r="F10">
+        <v>1.3492022862886328e-14</v>
+      </c>
+      <c r="G10">
+        <v>0.0</v>
+      </c>
+      <c r="H10">
+        <v>0.1446935496898365</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>-0.9921377386601338</v>
+      </c>
+      <c r="C11">
+        <v>0.0</v>
+      </c>
+      <c r="D11">
+        <v>-0.5204572812941508</v>
+      </c>
+      <c r="E11">
+        <v>-0.6168642282878078</v>
+      </c>
+      <c r="F11">
+        <v>1.3466694517385076e-14</v>
+      </c>
+      <c r="G11">
+        <v>0.0</v>
+      </c>
+      <c r="H11">
+        <v>0.12093144802170196</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>-0.931317131703341</v>
+      </c>
+      <c r="C12">
+        <v>0.0</v>
+      </c>
+      <c r="D12">
+        <v>-0.4780823352039434</v>
+      </c>
+      <c r="E12">
+        <v>-0.55652563000766</v>
+      </c>
+      <c r="F12">
+        <v>1.3412000973304146e-14</v>
+      </c>
+      <c r="G12">
+        <v>0.0</v>
+      </c>
+      <c r="H12">
+        <v>0.0998197529172211</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>-0.8688979012157383</v>
+      </c>
+      <c r="C13">
+        <v>0.0</v>
+      </c>
+      <c r="D13">
+        <v>-0.4491432070574239</v>
+      </c>
+      <c r="E13">
+        <v>-0.5118835184227113</v>
+      </c>
+      <c r="F13">
+        <v>1.3332628271158423e-14</v>
+      </c>
+      <c r="G13">
+        <v>0.0</v>
+      </c>
+      <c r="H13">
+        <v>0.08122018743975679</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>-0.8077995380727567</v>
+      </c>
+      <c r="C14">
+        <v>0.0</v>
+      </c>
+      <c r="D14">
+        <v>-0.42862347099201664</v>
+      </c>
+      <c r="E14">
+        <v>-0.4777426740355558</v>
+      </c>
+      <c r="F14">
+        <v>1.323281052728338e-14</v>
+      </c>
+      <c r="G14">
+        <v>0.0</v>
+      </c>
+      <c r="H14">
+        <v>0.06496131838760731</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>-0.748840312416389</v>
+      </c>
+      <c r="C15">
+        <v>0.0</v>
+      </c>
+      <c r="D15">
+        <v>-0.4131736946282153</v>
+      </c>
+      <c r="E15">
+        <v>-0.45057174710644904</v>
+      </c>
+      <c r="F15">
+        <v>1.3116338666312405e-14</v>
+      </c>
+      <c r="G15">
+        <v>0.0</v>
+      </c>
+      <c r="H15">
+        <v>0.05085802283126942</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>-0.6921339810602142</v>
+      </c>
+      <c r="C16">
+        <v>0.0</v>
+      </c>
+      <c r="D16">
+        <v>-0.40051669219830294</v>
+      </c>
+      <c r="E16">
+        <v>-0.427914314394589</v>
+      </c>
+      <c r="F16">
+        <v>1.2986577207574162e-14</v>
+      </c>
+      <c r="G16">
+        <v>0.0</v>
+      </c>
+      <c r="H16">
+        <v>0.038721943535952465</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>-0.6376112097334126</v>
+      </c>
+      <c r="C17">
+        <v>0.0</v>
+      </c>
+      <c r="D17">
+        <v>-0.38910425750697364</v>
+      </c>
+      <c r="E17">
+        <v>-0.40804913786530783</v>
+      </c>
+      <c r="F17">
+        <v>1.2846486722289322e-14</v>
+      </c>
+      <c r="G17">
+        <v>0.0</v>
+      </c>
+      <c r="H17">
+        <v>0.028367498022024082</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>-0.5851956049270015</v>
+      </c>
+      <c r="C18">
+        <v>0.0</v>
+      </c>
+      <c r="D18">
+        <v>-0.37790515148182624</v>
+      </c>
+      <c r="E18">
+        <v>-0.38978034641269066</v>
+      </c>
+      <c r="F18">
+        <v>1.2698650042513726e-14</v>
+      </c>
+      <c r="G18">
+        <v>0.0</v>
+      </c>
+      <c r="H18">
+        <v>0.01961552912300906</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>-0.5348503251242726</v>
+      </c>
+      <c r="C19">
+        <v>0.0</v>
+      </c>
+      <c r="D19">
+        <v>-0.3662630979125017</v>
+      </c>
+      <c r="E19">
+        <v>-0.3722967723993606</v>
+      </c>
+      <c r="F19">
+        <v>1.2545300696393843e-14</v>
+      </c>
+      <c r="G19">
+        <v>0.0</v>
+      </c>
+      <c r="H19">
+        <v>0.012295576831407232</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>-0.48657969434858706</v>
+      </c>
+      <c r="C20">
+        <v>0.0</v>
+      </c>
+      <c r="D20">
+        <v>-0.35379549635818497</v>
+      </c>
+      <c r="E20">
+        <v>-0.3550714206232398</v>
+      </c>
+      <c r="F20">
+        <v>1.2388352375174012e-14</v>
+      </c>
+      <c r="G20">
+        <v>0.0</v>
+      </c>
+      <c r="H20">
+        <v>0.00624726656368428</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>-0.44041765856436416</v>
+      </c>
+      <c r="C21">
+        <v>0.0</v>
+      </c>
+      <c r="D21">
+        <v>-0.3403183431064198</v>
+      </c>
+      <c r="E21">
+        <v>-0.3377867288833952</v>
+      </c>
+      <c r="F21">
+        <v>1.2229428513066768e-14</v>
+      </c>
+      <c r="G21">
+        <v>0.0</v>
+      </c>
+      <c r="H21">
+        <v>0.0013210919840288618</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
+  <dimension ref="A1:K21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>-3.452818634558829</v>
+      </c>
+      <c r="C2">
+        <v>0.0</v>
+      </c>
+      <c r="D2">
+        <v>-1.0</v>
+      </c>
+      <c r="E2">
+        <v>-0.6724381448767068</v>
+      </c>
+      <c r="F2">
+        <v>-8.622736026215812e-15</v>
+      </c>
+      <c r="G2">
+        <v>0.4586028719414287</v>
+      </c>
+      <c r="H2">
+        <v>-0.29161085716791146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>-2.247026625155925</v>
+      </c>
+      <c r="C3">
+        <v>0.0</v>
+      </c>
+      <c r="D3">
+        <v>-1.0</v>
+      </c>
+      <c r="E3">
+        <v>-0.6754920439440939</v>
+      </c>
+      <c r="F3">
+        <v>-9.136479065758198e-15</v>
+      </c>
+      <c r="G3">
+        <v>0.2231931345543115</v>
+      </c>
+      <c r="H3">
+        <v>-0.33915754479466115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>-1.6205323788595911</v>
+      </c>
+      <c r="C4">
+        <v>0.0</v>
+      </c>
+      <c r="D4">
+        <v>-1.0</v>
+      </c>
+      <c r="E4">
+        <v>-0.691426733217315</v>
+      </c>
+      <c r="F4">
+        <v>-9.571849997976843e-15</v>
+      </c>
+      <c r="G4">
+        <v>0.17337718670339702</v>
+      </c>
+      <c r="H4">
+        <v>-0.335995537700286</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>-1.2672896844330854</v>
+      </c>
+      <c r="C5">
+        <v>0.0</v>
+      </c>
+      <c r="D5">
+        <v>-1.0</v>
+      </c>
+      <c r="E5">
+        <v>-0.7126190796009915</v>
+      </c>
+      <c r="F5">
+        <v>-9.933327023769615e-15</v>
+      </c>
+      <c r="G5">
+        <v>0.13606624062531958</v>
+      </c>
+      <c r="H5">
+        <v>-0.3194967604267933</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>-1.0342703989673772</v>
+      </c>
+      <c r="C6">
+        <v>0.0</v>
+      </c>
+      <c r="D6">
+        <v>-0.9999999999999999</v>
+      </c>
+      <c r="E6">
+        <v>-0.7369490309361169</v>
+      </c>
+      <c r="F6">
+        <v>-1.022616636842296e-14</v>
+      </c>
+      <c r="G6">
+        <v>0.10077323633482829</v>
+      </c>
+      <c r="H6">
+        <v>-0.29755420498113316</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>-0.8446534793547625</v>
+      </c>
+      <c r="C7">
+        <v>0.0</v>
+      </c>
+      <c r="D7">
+        <v>-0.9999999999999998</v>
+      </c>
+      <c r="E7">
+        <v>-0.7634137716033644</v>
+      </c>
+      <c r="F7">
+        <v>-1.0456084872095713e-14</v>
+      </c>
+      <c r="G7">
+        <v>2.063782970431291</v>
+      </c>
+      <c r="H7">
+        <v>-0.27236297336874193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>-0.658731170928402</v>
+      </c>
+      <c r="C8">
+        <v>0.0</v>
+      </c>
+      <c r="D8">
+        <v>1.0018733440900165</v>
+      </c>
+      <c r="E8">
+        <v>1.2106152491219961</v>
+      </c>
+      <c r="F8">
+        <v>-1.062900957022899e-14</v>
+      </c>
+      <c r="G8">
+        <v>0.0</v>
+      </c>
+      <c r="H8">
+        <v>-0.2449613808818727</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0.24680905953848012</v>
+      </c>
+      <c r="C9">
+        <v>0.0</v>
+      </c>
+      <c r="D9">
+        <v>1.0184154340611102</v>
+      </c>
+      <c r="E9">
+        <v>1.1997204343437655</v>
+      </c>
+      <c r="F9">
+        <v>-1.0750883791106619e-14</v>
+      </c>
+      <c r="G9">
+        <v>0.0</v>
+      </c>
+      <c r="H9">
+        <v>-0.2161313684701008</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>0.7263675921425261</v>
+      </c>
+      <c r="C10">
+        <v>0.0</v>
+      </c>
+      <c r="D10">
+        <v>0.81565738323619</v>
+      </c>
+      <c r="E10">
+        <v>0.9711631474977502</v>
+      </c>
+      <c r="F10">
+        <v>-1.0827520518668891e-14</v>
+      </c>
+      <c r="G10">
+        <v>0.0</v>
+      </c>
+      <c r="H10">
+        <v>-0.18772319729265108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>0.8982855718353072</v>
+      </c>
+      <c r="C11">
+        <v>0.0</v>
+      </c>
+      <c r="D11">
+        <v>0.6586264335291755</v>
+      </c>
+      <c r="E11">
+        <v>0.7905470542901599</v>
+      </c>
+      <c r="F11">
+        <v>-1.0864494887789338e-14</v>
+      </c>
+      <c r="G11">
+        <v>0.0</v>
+      </c>
+      <c r="H11">
+        <v>-0.1610106683164092</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>0.925522701303046</v>
+      </c>
+      <c r="C12">
+        <v>0.0</v>
+      </c>
+      <c r="D12">
+        <v>0.55700364670584</v>
+      </c>
+      <c r="E12">
+        <v>0.6677310999777977</v>
+      </c>
+      <c r="F12">
+        <v>-1.0867068720641567e-14</v>
+      </c>
+      <c r="G12">
+        <v>0.0</v>
+      </c>
+      <c r="H12">
+        <v>-0.1365906107359131</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>0.89464697633588</v>
+      </c>
+      <c r="C13">
+        <v>0.0</v>
+      </c>
+      <c r="D13">
+        <v>0.49186589094681055</v>
+      </c>
+      <c r="E13">
+        <v>0.5837699848463282</v>
+      </c>
+      <c r="F13">
+        <v>-1.0840140977964427e-14</v>
+      </c>
+      <c r="G13">
+        <v>0.0</v>
+      </c>
+      <c r="H13">
+        <v>-0.11464720511777458</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>0.8432769678272422</v>
+      </c>
+      <c r="C14">
+        <v>0.0</v>
+      </c>
+      <c r="D14">
+        <v>0.44886422568029916</v>
+      </c>
+      <c r="E14">
+        <v>0.524200293667064</v>
+      </c>
+      <c r="F14">
+        <v>-1.0788218883580525e-14</v>
+      </c>
+      <c r="G14">
+        <v>0.0</v>
+      </c>
+      <c r="H14">
+        <v>-0.09515749882355043</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>0.78628418943233</v>
+      </c>
+      <c r="C15">
+        <v>0.0</v>
+      </c>
+      <c r="D15">
+        <v>0.41930366274779857</v>
+      </c>
+      <c r="E15">
+        <v>0.4801724794746719</v>
+      </c>
+      <c r="F15">
+        <v>-1.0715405280632185e-14</v>
+      </c>
+      <c r="G15">
+        <v>0.0</v>
+      </c>
+      <c r="H15">
+        <v>-0.07800296479348615</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>0.7291287172948269</v>
+      </c>
+      <c r="C16">
+        <v>0.0</v>
+      </c>
+      <c r="D16">
+        <v>0.397940575159894</v>
+      </c>
+      <c r="E16">
+        <v>0.4462730444426526</v>
+      </c>
+      <c r="F16">
+        <v>-1.0625398492454296e-14</v>
+      </c>
+      <c r="G16">
+        <v>0.0</v>
+      </c>
+      <c r="H16">
+        <v>-0.06302357283899464</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>0.6736313551308283</v>
+      </c>
+      <c r="C17">
+        <v>0.0</v>
+      </c>
+      <c r="D17">
+        <v>0.3814757938432244</v>
+      </c>
+      <c r="E17">
+        <v>0.41902976580951823</v>
+      </c>
+      <c r="F17">
+        <v>-1.0521501591329904e-14</v>
+      </c>
+      <c r="G17">
+        <v>0.0</v>
+      </c>
+      <c r="H17">
+        <v>-0.05004343869535837</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>0.6202949310831299</v>
+      </c>
+      <c r="C18">
+        <v>0.0</v>
+      </c>
+      <c r="D18">
+        <v>0.36775375988496617</v>
+      </c>
+      <c r="E18">
+        <v>0.39611715994926344</v>
+      </c>
+      <c r="F18">
+        <v>-1.0406638528335869e-14</v>
+      </c>
+      <c r="G18">
+        <v>0.0</v>
+      </c>
+      <c r="H18">
+        <v>-0.03888338257389103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>0.5691926844693456</v>
+      </c>
+      <c r="C19">
+        <v>0.0</v>
+      </c>
+      <c r="D19">
+        <v>0.3553437873111153</v>
+      </c>
+      <c r="E19">
+        <v>0.37594124158524256</v>
+      </c>
+      <c r="F19">
+        <v>-1.0283375052422972e-14</v>
+      </c>
+      <c r="G19">
+        <v>0.0</v>
+      </c>
+      <c r="H19">
+        <v>-0.029367464426564148</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>0.5202897774842203</v>
+      </c>
+      <c r="C20">
+        <v>0.0</v>
+      </c>
+      <c r="D20">
+        <v>0.3433055700353689</v>
+      </c>
+      <c r="E20">
+        <v>0.3574070387942728</v>
+      </c>
+      <c r="F20">
+        <v>-1.0153942753091595e-14</v>
+      </c>
+      <c r="G20">
+        <v>0.0</v>
+      </c>
+      <c r="H20">
+        <v>-0.021326604155422448</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>0.4735483412482155</v>
+      </c>
+      <c r="C21">
+        <v>0.0</v>
+      </c>
+      <c r="D21">
+        <v>0.33104442188153804</v>
+      </c>
+      <c r="E21">
+        <v>0.3397749693612522</v>
+      </c>
+      <c r="F21">
+        <v>-1.0020264905286315e-14</v>
+      </c>
+      <c r="G21">
+        <v>0.0</v>
+      </c>
+      <c r="H21">
+        <v>-0.014600660752960591</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Draft v2 prepared and checked
</commit_message>
<xml_diff>
--- a/irf/irf/Paper IRFs.xlsx
+++ b/irf/irf/Paper IRFs.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="143">
   <si>
     <t>t</t>
   </si>
@@ -437,6 +437,30 @@
   </si>
   <si>
     <t>2026-03-07T12:50:40.745</t>
+  </si>
+  <si>
+    <t>2026-03-08T23:41:18.378</t>
+  </si>
+  <si>
+    <t>2026-03-08T23:41:45.068</t>
+  </si>
+  <si>
+    <t>2026-03-08T23:41:51.843</t>
+  </si>
+  <si>
+    <t>2026-03-08T23:41:55.452</t>
+  </si>
+  <si>
+    <t>2026-03-08T23:41:59.378</t>
+  </si>
+  <si>
+    <t>2026-03-08T23:42:03.115</t>
+  </si>
+  <si>
+    <t>2026-03-08T23:42:07.443</t>
+  </si>
+  <si>
+    <t>2026-03-09T09:21:01.743</t>
   </si>
 </sst>
 </file>
@@ -2573,7 +2597,7 @@
         <v>5</v>
       </c>
       <c r="K1" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -3135,7 +3159,7 @@
         <v>5</v>
       </c>
       <c r="K1" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -3697,7 +3721,7 @@
         <v>5</v>
       </c>
       <c r="K1" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:11">

</xml_diff>

<commit_message>
Charting updates - CY trend added to FINAL counterfactual charts and Paper_IRF_charts_combined.jl is updated.
</commit_message>
<xml_diff>
--- a/irf/irf/Paper IRFs.xlsx
+++ b/irf/irf/Paper IRFs.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="425">
   <si>
     <t>t</t>
   </si>
@@ -1247,6 +1247,69 @@
   </si>
   <si>
     <t>2026-04-20T17:29:01.142</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:21:38.785</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:21:43.994</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:21:45.008</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:21:45.954</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:21:47.68</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:21:54.791</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:21:58.443</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:36:48.938</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:36:53.714</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:36:54.577</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:36:55.324</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:36:57.045</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:37:07.914</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:37:17.177</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:49:52.318</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:49:57.115</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:49:57.913</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:49:58.613</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:50:00.184</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:50:12.908</t>
+  </si>
+  <si>
+    <t>2026-04-23T18:50:22.024</t>
   </si>
 </sst>
 </file>
@@ -3371,7 +3434,7 @@
         <v>5</v>
       </c>
       <c r="W1" t="s">
-        <v>399</v>
+        <v>422</v>
       </c>
     </row>
     <row r="2" spans="1:23">
@@ -6459,7 +6522,7 @@
         <v>5</v>
       </c>
       <c r="K1" t="s">
-        <v>403</v>
+        <v>424</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -7021,7 +7084,7 @@
         <v>5</v>
       </c>
       <c r="K1" t="s">
-        <v>395</v>
+        <v>418</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -7612,7 +7675,7 @@
         <v>5</v>
       </c>
       <c r="K1" t="s">
-        <v>398</v>
+        <v>421</v>
       </c>
       <c r="L1" t="s">
         <v>163</v>

</xml_diff>